<commit_message>
aceite: a regua inteira na base completa, 165 de 165
- gerador/aceite.py e --aceite [--replica]: gera as seis etapas de ponta a
  ponta, confere cada uma, junta as medidas, conta as linhas na replica (tem
  de bater com o gerador, tabela a tabela) e passa a regua inteira. Medidas e
  laudo versionados em dados/regua, com README de como refazer e conferir.
- plausibilidade, sem mexer nos sorteios: o funil da etapa 3 passa a acontecer
  em horario comercial (30% das entrevistas caiam em fim de semana, a qualquer
  hora) por um mapa monotono da janela da vaga para o eixo do expediente; a
  assinatura de contrato comercial cai sempre em dia de semana.
- a base da etapa 4 carrega o gabarito das duplicatas (medida CAD-01).
- planilhas do consolidado regeneradas com a base nova.
- 6 testes: um deles gera tudo e prova que o laudo versionado e o da base que
  o gerador produz.
- higiene: .py e .md voltam a 644; so script fica executavel.
</commit_message>
<xml_diff>
--- a/dados/gerencial/consolidado_gerencial_2018.xlsx
+++ b/dados/gerencial/consolidado_gerencial_2018.xlsx
@@ -491,19 +491,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" t="n">
         <v>36</v>
       </c>
       <c r="E4" t="n">
-        <v>67668.3</v>
+        <v>71037.32000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>43250.86</v>
+        <v>45730.02</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>43144</v>
+        <v>43139</v>
       </c>
     </row>
     <row r="5">
@@ -522,13 +522,13 @@
         <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>184974.05</v>
+        <v>185872.63</v>
       </c>
       <c r="F5" t="n">
-        <v>111103.57</v>
+        <v>111965.21</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>43171</v>
+        <v>43167</v>
       </c>
     </row>
     <row r="6">
@@ -547,13 +547,13 @@
         <v>21</v>
       </c>
       <c r="E6" t="n">
-        <v>228664.06</v>
+        <v>227976.11</v>
       </c>
       <c r="F6" t="n">
-        <v>141042.87</v>
+        <v>139992.64</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>43203</v>
+        <v>43199</v>
       </c>
     </row>
     <row r="7">
@@ -572,13 +572,13 @@
         <v>31</v>
       </c>
       <c r="E7" t="n">
-        <v>262218.58</v>
+        <v>261808.06</v>
       </c>
       <c r="F7" t="n">
-        <v>157254.06</v>
+        <v>154942.12</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>43234</v>
+        <v>43228</v>
       </c>
     </row>
     <row r="8">
@@ -591,19 +591,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E8" t="n">
-        <v>253409.5</v>
+        <v>257684.63</v>
       </c>
       <c r="F8" t="n">
-        <v>148252.4</v>
+        <v>151752.95</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>43262</v>
+        <v>43264</v>
       </c>
     </row>
     <row r="9">
@@ -619,16 +619,16 @@
         <v>80</v>
       </c>
       <c r="D9" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E9" t="n">
-        <v>375811.28</v>
+        <v>375234.2</v>
       </c>
       <c r="F9" t="n">
-        <v>220587.54</v>
+        <v>218894.49</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>43294</v>
+        <v>43291</v>
       </c>
     </row>
     <row r="10">
@@ -644,16 +644,16 @@
         <v>92</v>
       </c>
       <c r="D10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" t="n">
-        <v>429942.45</v>
+        <v>430714.76</v>
       </c>
       <c r="F10" t="n">
-        <v>266430.42</v>
+        <v>267179.56</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>43322</v>
+        <v>43327</v>
       </c>
     </row>
     <row r="11">
@@ -672,13 +672,13 @@
         <v>39</v>
       </c>
       <c r="E11" t="n">
-        <v>444006.68</v>
+        <v>443824.58</v>
       </c>
       <c r="F11" t="n">
-        <v>289124.01</v>
+        <v>289838.38</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>43360</v>
+        <v>43354</v>
       </c>
     </row>
     <row r="12">
@@ -694,16 +694,16 @@
         <v>111</v>
       </c>
       <c r="D12" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E12" t="n">
-        <v>477952.71</v>
+        <v>478314.52</v>
       </c>
       <c r="F12" t="n">
-        <v>310373.12</v>
+        <v>310240.46</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>43388</v>
+        <v>43385</v>
       </c>
     </row>
     <row r="13">
@@ -722,10 +722,10 @@
         <v>36</v>
       </c>
       <c r="E13" t="n">
-        <v>564428.1800000001</v>
+        <v>564284.98</v>
       </c>
       <c r="F13" t="n">
-        <v>374121.05</v>
+        <v>373912.36</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>43413</v>
@@ -747,13 +747,13 @@
         <v>38</v>
       </c>
       <c r="E14" t="n">
-        <v>623370.88</v>
+        <v>623665.46</v>
       </c>
       <c r="F14" t="n">
-        <v>414478.16</v>
+        <v>415102.55</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>43444</v>
+        <v>43446</v>
       </c>
     </row>
     <row r="15">
@@ -769,13 +769,13 @@
         <v>151</v>
       </c>
       <c r="D15" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E15" t="n">
-        <v>679640.89</v>
+        <v>679693.6</v>
       </c>
       <c r="F15" t="n">
-        <v>445008.72</v>
+        <v>443787.34</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>43479</v>
@@ -788,13 +788,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E16" t="n">
-        <v>4592087.56</v>
+        <v>4600110.85</v>
       </c>
       <c r="F16" t="n">
-        <v>2921026.78</v>
+        <v>2923338.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>